<commit_message>
Merge empty spacer cells in the Benchmark Detail repeatability block
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DSsZtqnJz4gnTpb63ff5Gb
</commit_message>
<xml_diff>
--- a/Week5_Brightline_Tradeoff_Board.xlsx
+++ b/Week5_Brightline_Tradeoff_Board.xlsx
@@ -15698,7 +15698,7 @@
       <c r="A13" s="66" t="s">
         <v>99</v>
       </c>
-      <c r="B13" s="36"/>
+      <c r="B13" s="66"/>
       <c r="C13" s="67">
         <f>C5</f>
         <v>5.227630999968369</v>
@@ -15723,7 +15723,7 @@
       <c r="A14" s="66" t="s">
         <v>100</v>
       </c>
-      <c r="B14" s="36"/>
+      <c r="B14" s="66"/>
       <c r="C14" s="67">
         <f>D5</f>
         <v>6.531877149961926</v>
@@ -15802,8 +15802,11 @@
       <c r="O18" s="17"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="7">
     <mergeCell ref="A11:O11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
     <mergeCell ref="A15:O15"/>
     <mergeCell ref="A17:O17"/>
     <mergeCell ref="A18:O18"/>

</xml_diff>